<commit_message>
doc: I made Decision Log 4, also uploaded the interview record with the developer
</commit_message>
<xml_diff>
--- a/test/human_scores.xlsx
+++ b/test/human_scores.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>scored_at</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -483,12 +483,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -559,18 +559,18 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -666,12 +666,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -755,18 +755,18 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -844,12 +844,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -937,18 +937,18 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1035,12 +1035,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1109,18 +1109,18 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>selim</t>
+          <t>HEY HEY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-04-12T13:56:56</t>
+          <t>2026-04-13T13:09:08</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1211,6 +1211,737 @@
         <v>2</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Question:
+Why am I getting a segmentation fault when accessing an array in C?
+Code:
+#include &lt;stdio.h&gt;
+int main() {
+    int *arr;
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Answer A</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Frontier proprietary model</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>gpt-5.4</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>`arr` is a pointer, but it does not point to valid memory.
+### What is wrong
+```c
+int *arr;
+arr[0] = 10;
+```
+Here, `arr` is an uninitialized pointer. It contains a garbage address, so writing to `arr[0]` tries to access memory you do not own. That causes a segmentation fault.
+### Correct fix
+Allocate valid memory for the pointer before using it.
+### Corrected code
+```c
+#include &lt;stdio.h&gt;
+#include &lt;stdlib.h&gt;
+int main() {
+    int *arr = malloc(sizeof(int));
+    if (arr == NULL) {
+        return 1;
+    }
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    free(arr);
+    return 0;
+}
+```
+### Summary
+You must make `arr` point to valid memory before indexing it. `malloc` gives you that memory, and `free` releases it when done.</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Question:
+Why am I getting a segmentation fault when accessing an array in C?
+Code:
+#include &lt;stdio.h&gt;
+int main() {
+    int *arr;
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Answer B</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Frontier competitor</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4-6</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>## The Problem
+`arr` is a **pointer that has never been initialized** — it contains a garbage memory address. Writing to `arr[0]` means writing to some random memory location, which causes a segmentation fault.
+---
+## What's Wrong
+```c
+int *arr;   // ⚠️ Uninitialized pointer — points to garbage address
+arr[0] = 10; // ❌ Writing to unknown memory → segfault
+```
+---
+## The Fix
+You need to either:
+- **Allocate memory dynamically** with `malloc`, or
+- **Use a stack-allocated array** directly
+### Option 1 — Dynamic allocation (heap)
+```c
+#include &lt;stdio.h&gt;
+#include &lt;stdlib.h&gt;
+int main() {
+    int *arr = malloc(5 * sizeof(int)); // Allocate space for 5 integers
+    if (arr == NULL) {                  // Always check malloc result
+        return 1;
+    }
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    free(arr); // Release memory when done
+    return 0;
+}
+```
+### Option 2 — Stack array (simpler for fixed sizes)
+```c
+#include &lt;stdio.h&gt;
+int main() {
+    int arr[5]; // Memory allocated automatically on the stack
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}
+```
+---
+## Key Takeaway
+| Approach | When to use |
+|---|---|
+| `int arr[N]` | Fixed, known size at compile time |
+| `malloc` | Dynamic or large sizes |
+&gt; **Always ensure a pointer points to valid, allocated memory before dereferencing it.**</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Question:
+Why am I getting a segmentation fault when accessing an array in C?
+Code:
+#include &lt;stdio.h&gt;
+int main() {
+    int *arr;
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Answer C</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Open-source model</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>openrouter</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-maverick</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t># Step-by-step analysis of the problem:
+1. **The code declares a pointer `arr` to an integer**: The line `int *arr;` declares a pointer `arr` that is supposed to point to an integer. However, it does not allocate any memory for the integer.
+2. **The pointer is not initialized**: The pointer `arr` is not initialized to point to a valid memory location. It contains an indeterminate value, which is often referred to as a "garbage value."
+3. **Accessing the pointer as an array**: The line `arr[0] = 10;` attempts to access the memory location pointed to by `arr` as if it were an array. Since `arr` is not pointing to a valid memory location, this results in **undefined behavior**.
+4. **The undefined behavior manifests as a segmentation fault**: In this specific case, the undefined behavior results in a segmentation fault because the program is trying to access a memory location that it is not allowed to access.
+# Fixed solution:
+```c
+#include &lt;stdio.h&gt;
+#include &lt;stdlib.h&gt;
+int main() {
+    // Allocate memory for one integer
+    int *arr = malloc(sizeof(int));
+    if (arr == NULL) {
+        // Handle memory allocation failure
+        printf("Memory allocation failed\n");
+        return 1;
+    }
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    // Don't forget to free the allocated memory
+    free(arr);
+    return 0;
+}
+```
+# Explanation of changes:
+*   **Allocated memory for the pointer**: We used `malloc` to allocate memory for one integer and assigned the address of this memory to `arr`.
+*   **Checked for memory allocation failure**: We checked if `malloc` returned `NULL`, indicating that the memory allocation failed.
+*   **Freed the allocated memory**: We used `free` to release the allocated memory back to the system to prevent memory leaks.
+# Alternative solution:
+If you know the size of the array at compile time, you can declare it as a regular array instead of using a pointer and dynamic memory allocation:
+```c
+#include &lt;stdio.h&gt;
+int main() {
+    int arr[1];  // Declare an array of size 1
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}
+```</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Question:
+Why am I getting a segmentation fault when accessing an array in C?
+Code:
+#include &lt;stdio.h&gt;
+int main() {
+    int *arr;
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Answer D</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Budget / lightweight model</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>gpt-5.4-mini</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>The segmentation fault happens because `arr` is an uninitialized pointer.
+### 1. Explain the problem
+```c
+int *arr;
+```
+This declares a pointer, but it does **not** point to valid memory yet.  
+So when you do:
+```c
+arr[0] = 10;
+```
+you are writing to an invalid location, which causes undefined behavior and usually a segmentation fault.
+### 2. What is wrong
+- `arr` has no allocated memory
+- You are using `arr[0]` before assigning `arr` to valid storage
+### 3. Correct solution
+Allocate memory for the array before using it. For one `int`, you can use a real array or dynamically allocate memory. The simplest fix here is to use a normal array.
+### 4. Corrected code
+```c
+#include &lt;stdio.h&gt;
+int main() {
+    int arr[1];
+    arr[0] = 10;
+    printf("%d\n", arr[0]);
+    return 0;
+}
+```
+If you want, I can also show the `malloc` version.</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Question:
+Why is my string not changing after passing it to a function in C?
+Code:
+#include &lt;stdio.h&gt;
+void changeString(char str[]) {
+    str = "Hello";
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Answer A</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Frontier proprietary model</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>gpt-5.4</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>`str` is not changing because inside `changeString`, you are only changing the local pointer parameter, not the contents of the original array.
+### What is wrong
+In this function:
+```c
+void changeString(char str[]) {
+    str = "Hello";
+}
+```
+`str` behaves like a local pointer (`char *str`). Assigning:
+```c
+str = "Hello";
+```
+only makes that local pointer point to `"Hello"`. It does **not** copy `"Hello"` into the array in `main`.
+So `main` still has:
+```c
+char str[] = "World";
+```
+and that is what gets printed.
+---
+### Correct solution
+If you want to change the actual contents of the array, copy the new string into it with `strcpy`.
+### Corrected code
+```c
+#include &lt;stdio.h&gt;
+#include &lt;string.h&gt;
+void changeString(char str[]) {
+    strcpy(str, "Hello");
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}
+```
+### Output
+```c
+Hello
+```
+Make sure the destination array is large enough for the new string and the null terminator. In this case, `"World"` and `"Hello"` are both 5 characters, so it fits.</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Question:
+Why is my string not changing after passing it to a function in C?
+Code:
+#include &lt;stdio.h&gt;
+void changeString(char str[]) {
+    str = "Hello";
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Answer B</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Frontier competitor</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4-6</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>## The Problem
+Inside `changeString()`, you're reassigning the **local pointer** `str` to point to a string literal — this has no effect on the original array in `main()`.
+When an array is passed to a function, it **decays into a pointer**. Reassigning that pointer only changes the local copy; the original array in `main()` is untouched.
+```c
+void changeString(char str[]) {
+    str = "Hello";  // ❌ Only reassigns the local pointer, original unchanged
+}
+```
+---
+## The Fix
+Use `strcpy()` to copy the string **contents** into the existing array's memory location.
+---
+## Corrected Code
+```c
+#include &lt;stdio.h&gt;
+#include &lt;string.h&gt;
+void changeString(char str[]) {
+    strcpy(str, "Hello");  // ✅ Copies characters into the original array's memory
+}
+int main() {
+    char str[] = "World";  // Array is large enough to hold "Hello"
+    changeString(str);
+    printf("%s", str);     // Output: Hello
+    return 0;
+}
+```
+---
+## Key Points
+| Approach | What happens |
+|---|---|
+| `str = "Hello"` | Reassigns local pointer only — **no effect** outside |
+| `strcpy(str, "Hello")` | Writes into the actual memory — **works correctly** |
+&gt; ⚠️ **Important:** Ensure the destination array is large enough for the new string to avoid a buffer overflow. Here `"World"` (5 chars + `\0`) and `"Hello"` are the same size, so it's safe.</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Question:
+Why is my string not changing after passing it to a function in C?
+Code:
+#include &lt;stdio.h&gt;
+void changeString(char str[]) {
+    str = "Hello";
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Answer C</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Open-source model</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>openrouter</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-maverick</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>### Problem Explanation
+The issue here is that the string `str` in `main()` is not being modified after calling `changeString(str)`.
+### What's Wrong
+The problem lies in how C handles array passing to functions. When you pass an array to a function, it "decays" into a pointer to its first element. However, inside the function, this pointer is a local copy. So, when you do `str = "Hello";` inside `changeString`, you're changing the local pointer `str` to point to the string literal "Hello", not modifying the original array in `main()`.
+### Correct Solution
+To modify the original string, you should copy the new string into the array pointed to by `str`, rather than changing `str` to point to a different string. You can use `strcpy` from `string.h` to achieve this.
+### Corrected Code
+```c
+#include &lt;stdio.h&gt;
+#include &lt;string.h&gt;
+void changeString(char str[]) {
+    strcpy(str, "Hello"); // Copy "Hello" into the array pointed to by str
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}
+```
+This code will output "Hello" as expected. Note that using `strcpy` assumes that the destination buffer is large enough to hold the source string. In this case, it's safe because "Hello" is not longer than "World". Always ensure the buffer size is sufficient when using `strcpy` to avoid buffer overflows.</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HEY HEY</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-04-13T13:09:09</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Question:
+Why is my string not changing after passing it to a function in C?
+Code:
+#include &lt;stdio.h&gt;
+void changeString(char str[]) {
+    str = "Hello";
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Answer D</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Budget / lightweight model</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>gpt-5.4-mini</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1. **Explain the problem**
+In C, function arguments are passed **by value**.  
+That means `changeString(str)` receives a copy of the pointer to the array, not the original array itself.
+So this line:
+```c
+str = "Hello";
+```
+only changes the local copy of the pointer inside `changeString()`. It does **not** modify the contents of the string in `main()`.
+Also, `str` in `main()` is a writable character array, while `"Hello"` is a string literal. Assigning the pointer does not copy the text into the array.
+---
+2. **What is wrong**
+This is the wrong part:
+```c
+str = "Hello";
+```
+You are reassigning the local parameter instead of writing into the array.
+If you want to change the actual string contents, you must copy the characters into the array.
+---
+3. **Correct solution**
+Use `strcpy()` to copy `"Hello"` into the array.
+Since `str` in `main()` is an array, it has enough space for `"Hello"` only if the array is large enough. In your example, `"World"` is 6 bytes including the null terminator, which is enough for `"Hello"` too.
+---
+4. **Corrected code**
+```c
+#include &lt;stdio.h&gt;
+#include &lt;string.h&gt;
+void changeString(char str[]) {
+    strcpy(str, "Hello");
+}
+int main() {
+    char str[] = "World";
+    changeString(str);
+    printf("%s", str);
+    return 0;
+}
+```
+This will print:
+```c
+Hello
+```</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>